<commit_message>
"Completato" il convertitore da excel a sql (potrebbe cambiare quando verra implementato il database)
</commit_message>
<xml_diff>
--- a/DatiExcel/VetPortal_DatiImportazione.xlsx
+++ b/DatiExcel/VetPortal_DatiImportazione.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Istruzioni"/>
@@ -1423,7 +1423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1453,7 +1453,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1485,6 +1485,9 @@
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1493,6 +1496,9 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1800,7 +1806,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="10" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="60.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="25" width="60.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1816,25 +1822,25 @@
       <c r="B2" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="19"/>
+      <c r="A3" s="21"/>
       <c r="B3" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="22" t="s">
         <v>386</v>
       </c>
       <c r="B4" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="23" t="s">
         <v>387</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="23" t="s">
         <v>388</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="21" t="s">
         <v>389</v>
       </c>
       <c r="B6" s="19" t="s">
@@ -1842,7 +1848,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="21" t="s">
         <v>391</v>
       </c>
       <c r="B7" s="19" t="s">
@@ -1850,7 +1856,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="21" t="s">
         <v>393</v>
       </c>
       <c r="B8" s="19" t="s">
@@ -1858,7 +1864,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="21" t="s">
         <v>395</v>
       </c>
       <c r="B9" s="19" t="s">
@@ -1866,17 +1872,17 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="19"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="22" t="s">
         <v>397</v>
       </c>
       <c r="B11" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="21" t="s">
         <v>398</v>
       </c>
       <c r="B12" s="19" t="s">
@@ -1884,7 +1890,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="21" t="s">
         <v>400</v>
       </c>
       <c r="B13" s="19" t="s">
@@ -1892,7 +1898,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="21" t="s">
         <v>180</v>
       </c>
       <c r="B14" s="19" t="s">
@@ -1900,7 +1906,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="21" t="s">
         <v>403</v>
       </c>
       <c r="B15" s="19" t="s">
@@ -1908,7 +1914,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="21" t="s">
         <v>405</v>
       </c>
       <c r="B16" s="19" t="s">
@@ -1916,7 +1922,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="21" t="s">
         <v>407</v>
       </c>
       <c r="B17" s="19" t="s">
@@ -1924,11 +1930,11 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="19"/>
+      <c r="A18" s="21"/>
       <c r="B18" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="23"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="19"/>
     </row>
   </sheetData>

</xml_diff>